<commit_message>
docs: point the README and the sheet templates at Mastodon for currency
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/1_기본_상점_스탯.xlsx
+++ b/templates/1_기본_상점_스탯.xlsx
@@ -10,14 +10,9 @@
     <sheet name="설정" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="도움말" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="운영진 명령어" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="명단" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="관리" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="상점" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="운세" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="키워드" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="랜덤박스" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="출석부" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="기록" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="운세" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="키워드" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="랜덤박스" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -437,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -465,244 +460,67 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>재화 이름</t>
+          <t>하루 조사 횟수</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>코인</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>소지금 단위</t>
+          <t>하루 [조사] 횟수 (0 = 제한 없음)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>양도</t>
+          <t>랜덤박스 명령어</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>사용</t>
+          <t>랜덤박스</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>[양도] 명령어 (사용/미사용)</t>
+          <t>랜덤박스를 여는 명령어 이름</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>출석 보상</t>
+          <t>키워드 이미지</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>사용</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>[출석] 한 번에 주는 재화 (0 = 출석 끔)</t>
+          <t>키워드 답변 이미지 첨부 (사용/미사용)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>툿 보상 기준</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>운영진</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>툿 N개마다 재화 지급 (0 = 끔)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>툿 보상 재화</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>그때 주는 재화</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>하루 조사 횟수</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>하루 [조사] 횟수 (0 = 제한 없음)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>랜덤박스 명령어</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>랜덤박스</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>랜덤박스를 여는 명령어 이름</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>키워드 이미지</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>사용</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>키워드 답변 이미지 첨부 (사용/미사용)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>운영진</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr"/>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
           <t>운영진 아이디 (쉼표로 여러 명). 서버 설정의 운영진에 더해집니다</t>
         </is>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>날짜</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>시간</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>이름</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>아이디</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>시간</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>이름</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>아이디</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>종류</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>내용</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -714,7 +532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -816,202 +634,82 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>[가방]</t>
+          <t>[랜덤박스/박스명]</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>현재 소지금과 소지품을 확인합니다.</t>
+          <t>랜덤박스를 엽니다. [랜덤박스]는 박스 목록</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>[상점]</t>
+          <t>[장소 목록]</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>상점 목록을 출력합니다.</t>
+          <t>진입할 수 있는 장소 목록을 봅니다.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>[구매/아이템명]</t>
+          <t>[진입/장소명]</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>원하는 아이템을 구매합니다. [구매/아이템명/수량]도 가능</t>
+          <t>장소에 들어갑니다.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>[설명/아이템명]</t>
+          <t>[조사/포인트명]</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>아이템의 설명을 출력합니다.</t>
+          <t>지금 장소의 조사 포인트를 조사합니다.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>[소모/아이템명]</t>
+          <t>[쪽지시험]</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>인벤토리에서 아이템을 소모합니다. (스탯 반영 X)</t>
+          <t>오늘의 쪽지시험 점수를 확인합니다.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>[상태 확인]</t>
+          <t>[낚시]</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>소지금, 소지품, 스탯을 확인합니다.</t>
+          <t>강가에서 낚시합니다.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>[사용/아이템명]</t>
+          <t>[스킬]</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>아이템을 사용합니다. (스탯 반영 O)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>[양도/n코인/캐릭터명]</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>n코인을 캐릭터에게 양도합니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>[양도/아이템명/캐릭터명]</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>아이템을 캐릭터에게 양도합니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>[출석]</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>하루 한 번 출석 보상을 받습니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>[랜덤박스/박스명]</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>랜덤박스를 엽니다. [랜덤박스]는 박스 목록</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>[장소 목록]</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>진입할 수 있는 장소 목록을 봅니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>[진입/장소명]</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>장소에 들어갑니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>[조사/포인트명]</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>지금 장소의 조사 포인트를 조사합니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>[쪽지시험]</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>오늘의 쪽지시험 점수를 확인합니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>[낚시]</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>강가에서 낚시합니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>[스킬]</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>스킬을 사용합니다.</t>
         </is>
@@ -1028,7 +726,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1073,105 +771,32 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>[소지금 추가/금액/캐릭터명]</t>
+          <t>[스진/워크시트명]</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>캐릭터명은 쉼표로 여러 명, '전원'이면 모두</t>
+          <t>STORY 계정에 DM 으로 보내면 스토리 시트의 그 워크시트를 송출</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>[소지금 추가/10/겐지, 디바]</t>
+          <t>[스진/1일차]</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>[소지금 차감/금액/캐릭터명]</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr"/>
+          <t>[스진 중지]</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>진행 중인 스토리를 멈춥니다.</t>
+        </is>
+      </c>
       <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>[소지금 차감/10/전원]</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>[ㅇㅇ 변경/수치/캐릭터명]</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>관리 탭의 스탯을 바꿉니다. 수치에 주사위 가능</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>[체력 변경/-1d6/겐지]</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>[아이템 추가/템: n, 템: n/캐릭터명]</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr"/>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>[아이템 추가/사과: 2, 포도: 3/겐지]</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>[아이템 차감/템: n/캐릭터명]</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr"/>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>[아이템 차감/사과: 1/전원]</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>[스진/워크시트명]</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>STORY 계정에 DM 으로 보내면 스토리 시트의 그 워크시트를 송출</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>[스진/1일차]</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>[스진 중지]</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>진행 중인 스토리를 멈춥니다.</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>[스진 중지]</t>
         </is>
@@ -1183,556 +808,6 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>이름</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>아이디</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>운영자</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>manager</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>엘레나</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Elena</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>소피아</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Sophia</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>루카스</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Lucas</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>마야</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Maya</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>그레이스</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Grace</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="4" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>이름</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>아이디</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr"/>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>소지금</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>소지품</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>체력</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>정신력</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>운영자</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>manager</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>바나나: 2, 사과: 1</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>90</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>엘레나</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Elena</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>반지: 1</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>86</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>소피아</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Sophia</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>아몬드: 2, 파란 꽃병: 1</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>63</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>54</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>루카스</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Lucas</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>48</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>마야</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Maya</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>91</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>93</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>그레이스</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Grace</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>84</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>59</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>아이템명</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>가격</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>설명</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>스탯</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>수치</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>반지</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>노란색 보석이 박힌 은색 반지다.</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>정신력</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>동화책</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>아이들이 읽을 법한 귀여운 동화책이다.</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>체력</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>사과</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>아삭아삭!</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>체력</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>1d10</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>바나나</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>부드럽고 달콤하고...</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>정신력</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>-(1d6+3)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>아몬드</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>비매품</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>사실은 청산가리입니다.</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>정신력</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>-20</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>파란 꽃병</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>꽃을 꽂아둘 수 있습니다.</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>사용 불가</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1812,7 +887,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2134,7 +1209,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>